<commit_message>
Update CSL holding to 3450 shares; include backlog of daily EOD reports
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260616.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260616.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.6</v>
+        <v>1.575</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.09</v>
+        <v>0.065</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.96%</t>
+          <t>4.30%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>245089.6</v>
+        <v>241260.07</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>13786.29</v>
+        <v>9956.76</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1.572</v>
+        <v>1.59</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.017</v>
+        <v>0.035</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.09%</t>
+          <t>2.25%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>110040</v>
+        <v>111300</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>1190</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="6">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>65.01000000000001</v>
+        <v>65.19</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.17</v>
+        <v>0.01</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-0.26%</t>
+          <t>0.02%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>9000</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>585090</v>
+        <v>586710</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-1530</v>
+        <v>90</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>160.715</v>
+        <v>161.88</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-1.075</v>
+        <v>0.09</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.66%</t>
+          <t>0.06%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.7</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-1.43%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>7000</v>
+        <v>6900</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>105.74</v>
+        <v>106.25</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.21</v>
+        <v>0.72</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.20%</t>
+          <t>0.68%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>3000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>317220</v>
+        <v>318750</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>630</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.23</v>
+        <v>0.25</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.025</v>
+        <v>-0.005</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-9.80%</t>
+          <t>-1.96%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>4600</v>
+        <v>5000</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-500</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="13">
@@ -731,24 +731,24 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>-0.002</v>
+        <v>0</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
         <v>700000</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0</v>
+        <v>1400</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>-1400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.105</v>
+        <v>0.1</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0</v>
+        <v>-0.005</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-4.76%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>988.26</v>
+        <v>941.2</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0</v>
+        <v>-47.06</v>
       </c>
     </row>
     <row r="15">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0.105</v>
+        <v>0.11</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.005</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-4.55%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>630</v>
+        <v>660</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-30</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>35.095</v>
+        <v>35.75</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.225</v>
+        <v>0.43</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.64%</t>
+          <t>1.22%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>30.005</v>
+        <v>30.04</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.545</v>
+        <v>0.58</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.85%</t>
+          <t>1.97%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>38646.44</v>
+        <v>38691.52</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>701.96</v>
+        <v>747.04</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1383888.77</v>
+        <v>1386197.26</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>12560.96</v>
+        <v>14869.45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>